<commit_message>
Updated the homepage layout and added new CSS
</commit_message>
<xml_diff>
--- a/Parking_info.xlsx
+++ b/Parking_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2883a816ce5198e/Documents/New project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="182" documentId="8_{BF5B5FC1-64AA-4606-A780-2BA5CC58300E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7FE4595-6D19-4AD3-882C-02AA3B7AD300}"/>
+  <xr:revisionPtr revIDLastSave="231" documentId="8_{BF5B5FC1-64AA-4606-A780-2BA5CC58300E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5614BAF-8CB3-4960-A411-A5C4D1383253}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CBAF2CAF-A10F-4227-9339-64D5C6E0372A}"/>
+    <workbookView xWindow="2330" yWindow="1130" windowWidth="14400" windowHeight="8170" xr2:uid="{CBAF2CAF-A10F-4227-9339-64D5C6E0372A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>17/04/2026</t>
   </si>
@@ -88,6 +88,18 @@
   </si>
   <si>
     <t>E20</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>36F-888.88</t>
+  </si>
+  <si>
+    <t>Gate</t>
+  </si>
+  <si>
+    <t>D18</t>
   </si>
 </sst>
 </file>
@@ -95,7 +107,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-409]h:mm\ AM/PM;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]h:mm\ AM/PM;@"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -162,7 +174,7 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -483,16 +495,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6638512A-F4C8-4887-974D-A2A2F408FE7D}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.90625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="2"/>
+    <col min="5" max="5" width="8.7265625" style="2"/>
+    <col min="6" max="6" width="7.81640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="10.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:7">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -508,149 +523,220 @@
       <c r="E1" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="14.5" thickBot="1">
-      <c r="A2" s="3" t="s">
+      <c r="F1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A2" s="3">
+        <v>46239</v>
+      </c>
+      <c r="B2" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B3" s="4">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C3" s="4">
         <v>0.54166666666666663</v>
       </c>
-      <c r="D2" s="1">
-        <f t="shared" ref="D2:D9" si="0">IF(C2&lt;TIME(18,0,0),2000,IF(C2&lt;=TIME(22,0,0),3000,""))</f>
+      <c r="D3" s="1">
+        <f t="shared" ref="D3:D10" si="0">IF(C3&lt;TIME(18,0,0),2000,IF(C3&lt;=TIME(22,0,0),3000,""))</f>
         <v>2000</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="14.5" thickBot="1">
-      <c r="A3" s="3" t="s">
+      <c r="F3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
+      <c r="G3" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4">
         <v>0.5</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C4" s="4">
         <v>0.75138888888888888</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D4" s="1">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="14.5" thickBot="1">
-      <c r="A4" s="3" t="s">
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B5" s="4">
         <v>0.41666666666666669</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C5" s="4">
         <v>0.5</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D5" s="1">
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="14.5" thickBot="1">
-      <c r="A5" s="3" t="s">
+      <c r="F5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="4">
+      <c r="G5" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4">
         <v>0</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C6" s="4">
         <v>0.75347222222222221</v>
-      </c>
-      <c r="D5" s="1">
-        <f t="shared" si="0"/>
-        <v>3000</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="14.5" thickBot="1">
-      <c r="A6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0.8041666666666667</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="14.5" thickBot="1">
-      <c r="A7" s="3">
-        <v>46360</v>
+        <v>13</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
       </c>
       <c r="B7" s="4">
-        <v>0.58333333333333337</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="C7" s="4">
-        <v>0.68888888888888888</v>
+        <v>0.8041666666666667</v>
       </c>
       <c r="D7" s="1">
         <f t="shared" si="0"/>
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.5" thickBot="1">
+        <v>14</v>
+      </c>
+      <c r="F7" s="2">
+        <v>3</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="14.5" thickBot="1">
       <c r="A8" s="3">
-        <v>46330</v>
+        <v>46360</v>
       </c>
       <c r="B8" s="4">
-        <v>0.29166666666666669</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="C8" s="4">
-        <v>0.74444444444444446</v>
+        <v>0.68888888888888888</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="14.5" thickBot="1">
+        <v>15</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="14.5" thickBot="1">
       <c r="A9" s="3">
-        <v>46299</v>
+        <v>46330</v>
       </c>
       <c r="B9" s="4">
         <v>0.29166666666666669</v>
       </c>
       <c r="C9" s="4">
-        <v>0.75</v>
+        <v>0.74444444444444446</v>
       </c>
       <c r="D9" s="1">
         <f t="shared" si="0"/>
+        <v>2000</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="2">
+        <v>3</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="14.5" thickBot="1">
+      <c r="A10" s="3">
+        <v>46299</v>
+      </c>
+      <c r="B10" s="4">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="D10" s="1">
+        <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>17</v>
+      </c>
+      <c r="F10" s="2">
+        <v>2</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>